<commit_message>
Porting plan and list: brought up to date with the regions restructuring
Filter/Sort ROIs, Regions to column, Column to ROIs, ROI annotation,
DBSCAN and per_region measurements are marked done; the remaining work is
recast for the new contract (measurements as per_region plugins, tracks
and MINFLUX traces as id columns).  The spreadsheet's annotation columns
are untouched; a column 'Update 2026-10-14' and a row for ROI annotation
are added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4rjWo2i91xceLvMFCkyKa
</commit_message>
<xml_diff>
--- a/docs/smap_porting/SMAP_porting_list.xlsx
+++ b/docs/smap_porting/SMAP_porting_list.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Port list'!$A$1:$N$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Port list'!$A$1:$O$156</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -54,7 +54,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +86,21 @@
         <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -114,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -148,6 +163,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -514,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N155"/>
+  <dimension ref="A1:O156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="7.6640625" customWidth="1" min="3" max="3"/>
@@ -524,6 +548,7 @@
     <col width="20.5" customWidth="1" style="13" min="10" max="10"/>
     <col width="21.83203125" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -597,6 +622,11 @@
           <t>Work package (plan)</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Update 2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -618,7 +648,7 @@
           <t>read TIFF / MM stacks, ADU→photons</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -664,7 +694,7 @@
           <t>fit many stacks in a row</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -710,7 +740,7 @@
           <t>several channels on one chip</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -760,7 +790,7 @@
           <t>DoG/Gauss filter, local max, cutoffs</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -906,7 +936,7 @@
           <t>fit only inside / exclude drawn regions of the chip</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -964,7 +994,7 @@
           <t>cut ROIs</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1010,7 +1040,7 @@
           <t>sum frames of one blink before fitting</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1060,7 +1090,7 @@
           <t>Gaussian / spline MLE (GPU)</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1184,7 +1214,7 @@
           <t>multi-channel global fit</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1230,7 +1260,7 @@
           <t>4Pi</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1284,7 +1314,7 @@
           <t>multi-emitter-aware single fitter</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1334,7 +1364,7 @@
           <t>deep-learning localization</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1396,7 +1426,7 @@
           <t>other high-density localizers</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1442,7 +1472,7 @@
           <t>fast non-MLE localizer</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1538,7 +1568,7 @@
           <t>filter before saving</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -1588,7 +1618,7 @@
           <t>live view, preview</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1630,7 +1660,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1742,7 +1772,7 @@
           <t>cspline PSF from beads</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1788,7 +1818,7 @@
           <t>PSF by inverse modelling</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1846,7 +1876,7 @@
           <t>fitted vs true bead z</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -1892,7 +1922,7 @@
           <t>depth-dependent PSF / z-scaling correction (Li et al. 2018)</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -1954,7 +1984,7 @@
           <t>camera gain/offset from data (Heintzmann 2016)</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2016,7 +2046,7 @@
           <t>channel intensity ratios / field dependence</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -2062,7 +2092,7 @@
           <t>double-helix PSF</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2120,7 +2150,7 @@
           <t>supercritical-angle z</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2162,7 +2192,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2208,7 +2238,7 @@
           <t>cross-correlation drift, x/y/z</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -2254,7 +2284,7 @@
           <t>show saved drift</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F34" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -2300,7 +2330,7 @@
           <t>fiducial-based drift</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2358,7 +2388,7 @@
           <t>apply drift of file A to file B (e.g. second channel)</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2416,7 +2446,7 @@
           <t>apply Picasso drift file</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2474,7 +2504,7 @@
           <t>entropy-based drift (DME)</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F38" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2520,7 +2550,7 @@
           <t>drift + magnification change</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F39" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2578,7 +2608,7 @@
           <t>transformation from localizations (beads, ratiometric)</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="F40" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -2640,7 +2670,7 @@
           <t>apply a transform to the localizations of one channel/file, merge paired locs</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F41" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2706,7 +2736,7 @@
           <t>shift between two layers by cross-correlation</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F42" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2768,7 +2798,7 @@
           <t>relative drift between channels vs frame</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F43" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2822,7 +2852,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F44" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2868,7 +2898,7 @@
           <t>stitch z-stacks of slabs into whole-cell 3D</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F45" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -2926,7 +2956,7 @@
           <t>colour from intensity ratio</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3034,7 +3064,7 @@
           <t>&gt;2 dyes from ratios</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F48" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3092,14 +3122,14 @@
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F49" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Auto, SMAP, csv, MINFLUX, smappy HDF5</t>
+          <t>File/Load/Auto: smappy HDF5, SMAP, MINFLUX, csv</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3117,6 +3147,11 @@
       <c r="L49" s="4" t="n"/>
       <c r="M49" s="4" t="n"/>
       <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>one loader now (File/Load/Auto) with a format choice</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -3138,7 +3173,7 @@
           <t>associate a widefield TIFF</t>
         </is>
       </c>
-      <c r="F50" s="3" t="inlineStr">
+      <c r="F50" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3184,7 +3219,7 @@
           <t>GUI settings</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F51" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3230,7 +3265,7 @@
           <t>DECODE output</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3265,6 +3300,11 @@
       <c r="N52" s="2" t="inlineStr">
         <is>
           <t>A2 Loaders</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>smaller now: a Reader in io/formats.py, not a plugin</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3328,7 @@
           <t>not in SMAP</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F53" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3323,6 +3363,11 @@
       <c r="N53" s="2" t="inlineStr">
         <is>
           <t>A2 Loaders</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>smaller now: a Reader in io/formats.py, not a plugin</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3391,7 @@
           <t>CSV/TXT/XLS, chosen columns, all or filtered</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F54" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3400,7 +3445,7 @@
           <t>Picasso format</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F55" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3458,7 +3503,7 @@
           <t>save _sml.mat</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3512,7 +3557,7 @@
           <t>rendered image as TIFF</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F57" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3558,7 +3603,7 @@
           <t>3D viewers</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F58" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3604,7 +3649,7 @@
         </is>
       </c>
       <c r="E59" s="2" t="n"/>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F59" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3650,7 +3695,7 @@
           <t>site-explorer data</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3692,7 +3737,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n"/>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F61" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -3738,7 +3783,7 @@
           <t>new field from an expression</t>
         </is>
       </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="F62" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3780,7 +3825,7 @@
         </is>
       </c>
       <c r="E63" s="2" t="n"/>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F63" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3826,14 +3871,14 @@
           <t>apply a filter as a step</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F64" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Chain/Layers</t>
+          <t>Analysis/Process/Layers</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3851,6 +3896,11 @@
       <c r="L64" s="4" t="n"/>
       <c r="M64" s="4" t="n"/>
       <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>moved to Analysis/Process/Layers</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="2" t="n">
@@ -3872,7 +3922,7 @@
           <t>use other fields as x/y/z</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="F65" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -3918,7 +3968,7 @@
           <t>merge loaded files into one table</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="F66" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -3984,7 +4034,7 @@
           <t>grouped ↔ ungrouped coordinates</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F67" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -4046,7 +4096,7 @@
           <t>combine locs with the same value of any field</t>
         </is>
       </c>
-      <c r="F68" s="6" t="inlineStr">
+      <c r="F68" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4085,6 +4135,11 @@
       <c r="N68" s="2" t="inlineStr">
         <is>
           <t>J Later</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>measuring per id: done (block over any id column); collapsing a region into one row still open, see plan J</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4159,7 @@
         </is>
       </c>
       <c r="E69" s="2" t="n"/>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F69" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4162,7 +4217,7 @@
           <t>geometric edits</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr">
+      <c r="F70" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4224,7 +4279,7 @@
           <t>local mean/median/quantile of a field around each loc</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F71" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4282,7 +4337,7 @@
         </is>
       </c>
       <c r="E72" s="2" t="n"/>
-      <c r="F72" s="6" t="inlineStr">
+      <c r="F72" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4332,7 +4387,7 @@
         </is>
       </c>
       <c r="E73" s="2" t="n"/>
-      <c r="F73" s="3" t="inlineStr">
+      <c r="F73" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4378,7 +4433,7 @@
           <t>any field vs any other</t>
         </is>
       </c>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="F74" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4424,7 +4479,7 @@
           <t>shift a layer for display</t>
         </is>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="F75" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4486,7 +4541,7 @@
           <t>3D view, side view</t>
         </is>
       </c>
-      <c r="F76" s="3" t="inlineStr">
+      <c r="F76" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4532,7 +4587,7 @@
           <t>voxel rendering, export as stack</t>
         </is>
       </c>
-      <c r="F77" s="6" t="inlineStr">
+      <c r="F77" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4594,7 +4649,7 @@
           <t>Voronoi-density image</t>
         </is>
       </c>
-      <c r="F78" s="6" t="inlineStr">
+      <c r="F78" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4652,7 +4707,7 @@
           <t>raw frames, image tags</t>
         </is>
       </c>
-      <c r="F79" s="3" t="inlineStr">
+      <c r="F79" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4698,7 +4753,7 @@
           <t>re-point to moved raw data</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="F80" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -4744,7 +4799,7 @@
           <t>TIFF intensity at each loc / site</t>
         </is>
       </c>
-      <c r="F81" s="6" t="inlineStr">
+      <c r="F81" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4790,7 +4845,7 @@
         </is>
       </c>
       <c r="E82" s="2" t="n"/>
-      <c r="F82" s="6" t="inlineStr">
+      <c r="F82" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -4848,7 +4903,7 @@
           <t>photons, precision, on-time</t>
         </is>
       </c>
-      <c r="F83" s="3" t="inlineStr">
+      <c r="F83" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4894,7 +4949,7 @@
           <t>FRC</t>
         </is>
       </c>
-      <c r="F84" s="3" t="inlineStr">
+      <c r="F84" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4940,7 +4995,7 @@
           <t>line profile with models</t>
         </is>
       </c>
-      <c r="F85" s="3" t="inlineStr">
+      <c r="F85" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -4986,7 +5041,7 @@
         </is>
       </c>
       <c r="E86" s="2" t="n"/>
-      <c r="F86" s="3" t="inlineStr">
+      <c r="F86" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -5036,7 +5091,7 @@
           <t>histogram + stats of any field</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
+      <c r="F87" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -5075,6 +5130,11 @@
       <c r="N87" s="2" t="inlineStr">
         <is>
           <t>A4 Histogram</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Regions/Summarize/Histograms = over regions; histogram of localizations still open (A4); make it per_region too</t>
         </is>
       </c>
     </row>
@@ -5098,7 +5158,7 @@
           <t>photons, locs, precision, bg … vs frame or file</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="F88" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -5164,7 +5224,7 @@
           <t>spectrum of x/y/z of beads</t>
         </is>
       </c>
-      <c r="F89" s="6" t="inlineStr">
+      <c r="F89" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5222,7 +5282,7 @@
           <t>decorrelation resolution</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
+      <c r="F90" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5264,7 +5324,7 @@
         </is>
       </c>
       <c r="E91" s="2" t="n"/>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="F91" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5322,12 +5382,16 @@
           <t>DBSCAN, cluster id per loc + cluster table</t>
         </is>
       </c>
-      <c r="F92" s="6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="G92" s="2" t="n"/>
+      <c r="F92" s="14" t="inlineStr">
+        <is>
+          <t>have</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Regions/Find/DBSCAN</t>
+        </is>
+      </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5361,6 +5425,11 @@
       <c r="N92" s="2" t="inlineStr">
         <is>
           <t>B2 Cluster</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>DONE: Analysis/Regions/Find/DBSCAN (cluster_id, n_in_cluster)</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5453,7 @@
           <t>Ripley's K/L/H, pair correlation (Sengupta 2011)</t>
         </is>
       </c>
-      <c r="F93" s="6" t="inlineStr">
+      <c r="F93" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5446,7 +5515,7 @@
           <t>Voronoi-cell density, clusters by threshold (SharpViSu)</t>
         </is>
       </c>
-      <c r="F94" s="6" t="inlineStr">
+      <c r="F94" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5481,6 +5550,11 @@
       <c r="N94" s="2" t="inlineStr">
         <is>
           <t>B1/B2 Neighbourhood + Cluster</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>open; as another Regions/Find plugin (B2) + density in Neighbourhood (B1)</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5578,7 @@
           <t>neighbours within r per loc</t>
         </is>
       </c>
-      <c r="F95" s="6" t="inlineStr">
+      <c r="F95" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5566,7 +5640,7 @@
           <t>random colour per cluster</t>
         </is>
       </c>
-      <c r="F96" s="6" t="inlineStr">
+      <c r="F96" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5605,6 +5679,11 @@
       <c r="N96" s="2" t="inlineStr">
         <is>
           <t>B2 Cluster</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>open; suggest a render/LUT option for any id column, not cluster-only</t>
         </is>
       </c>
     </row>
@@ -5628,12 +5707,16 @@
           <t>DBSCAN/k-means/GMM per site</t>
         </is>
       </c>
-      <c r="F97" s="6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="G97" s="2" t="n"/>
+      <c r="F97" s="15" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>block over cluster_id; no cluster-shape measure yet</t>
+        </is>
+      </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
           <t>P2</t>
@@ -5666,7 +5749,12 @@
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>B2 Cluster</t>
+          <t>B2b Cluster statistics</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>DONE by structure: block over cluster_id (nested in ROIs) with any per_region plugin; a cluster-shape measurement still open (B2b)</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5774,7 @@
         </is>
       </c>
       <c r="E98" s="2" t="n"/>
-      <c r="F98" s="6" t="inlineStr">
+      <c r="F98" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5732,7 +5820,7 @@
           <t>histogram of locs/blinks per cluster, fit with a model of protein number, maturation efficiency and re-activations</t>
         </is>
       </c>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="F99" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5771,6 +5859,11 @@
       <c r="N99" s="2" t="inlineStr">
         <is>
           <t>B4 Counting</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>clear path now: per_region measure + Summarize fit (like NPC Corners + labelling efficiency)</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5883,7 @@
         </is>
       </c>
       <c r="E100" s="2" t="n"/>
-      <c r="F100" s="3" t="inlineStr">
+      <c r="F100" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -5836,7 +5929,7 @@
           <t>link locs into tracks</t>
         </is>
       </c>
-      <c r="F101" s="6" t="inlineStr">
+      <c r="F101" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5875,6 +5968,11 @@
       <c r="N101" s="2" t="inlineStr">
         <is>
           <t>F SPT</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>tracks as an id column (track_id) -&gt; per_region plugins run per track for free</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5996,7 @@
           <t>MSD, diffusion coefficients, jump distances, track viewer</t>
         </is>
       </c>
-      <c r="F102" s="6" t="inlineStr">
+      <c r="F102" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -5937,6 +6035,11 @@
       <c r="N102" s="2" t="inlineStr">
         <is>
           <t>F SPT</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>analyses as per_region measures + summaries over tracks</t>
         </is>
       </c>
     </row>
@@ -5960,7 +6063,7 @@
           <t>external uTrack</t>
         </is>
       </c>
-      <c r="F103" s="6" t="inlineStr">
+      <c r="F103" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6006,7 +6109,7 @@
           <t>co-tracking, MINFLUX steps</t>
         </is>
       </c>
-      <c r="F104" s="6" t="inlineStr">
+      <c r="F104" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6041,6 +6144,11 @@
       <c r="N104" s="2" t="inlineStr">
         <is>
           <t>G MINFLUX</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>tid is already an id column -&gt; per-trace via regions</t>
         </is>
       </c>
     </row>
@@ -6064,14 +6172,14 @@
         </is>
       </c>
       <c r="E105" s="2" t="n"/>
-      <c r="F105" s="3" t="inlineStr">
+      <c r="F105" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Segment/NPC</t>
+          <t>Regions/Find/NPC</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -6101,6 +6209,11 @@
           <t>E3 Segmenter</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>finders and clusterers are one kind now (Regions/Find); presets still open</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="42" customHeight="1">
       <c r="A106" s="2" t="n">
@@ -6122,14 +6235,14 @@
         </is>
       </c>
       <c r="E106" s="2" t="n"/>
-      <c r="F106" s="3" t="inlineStr">
+      <c r="F106" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Density Peaks</t>
+          <t>Regions/Find/Density Peaks</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -6159,6 +6272,11 @@
           <t>E3 Segmenter</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Regions/Find/Density Peaks; presets / one-vs-many plugins still open</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="2" t="n">
@@ -6180,7 +6298,7 @@
         </is>
       </c>
       <c r="E107" s="2" t="n"/>
-      <c r="F107" s="6" t="inlineStr">
+      <c r="F107" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6215,6 +6333,11 @@
       <c r="N107" s="2" t="inlineStr">
         <is>
           <t>E1 ROI housekeeping</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>open; could be a Filter ROIs condition on position</t>
         </is>
       </c>
     </row>
@@ -6238,7 +6361,7 @@
         </is>
       </c>
       <c r="E108" s="2" t="n"/>
-      <c r="F108" s="6" t="inlineStr">
+      <c r="F108" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6273,6 +6396,11 @@
       <c r="N108" s="2" t="inlineStr">
         <is>
           <t>E1 ROI housekeeping</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>open; suggest a third region choice of Remove Localizations; for clusters a filter cluster_id&gt;0 does it</t>
         </is>
       </c>
     </row>
@@ -6296,14 +6424,14 @@
         </is>
       </c>
       <c r="E109" s="2" t="n"/>
-      <c r="F109" s="6" t="inlineStr">
-        <is>
-          <t>missing</t>
+      <c r="F109" s="15" t="inlineStr">
+        <is>
+          <t>partly</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>(no cells)</t>
+          <t>Column to ROIs on filenumber</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -6329,6 +6457,11 @@
       <c r="L109" s="4" t="n"/>
       <c r="M109" s="4" t="n"/>
       <c r="N109" s="2" t="inlineStr"/>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>mostly there: Column to ROIs on filenumber</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="56" customHeight="1">
       <c r="A110" s="2" t="n">
@@ -6350,7 +6483,7 @@
         </is>
       </c>
       <c r="E110" s="2" t="n"/>
-      <c r="F110" s="4" t="inlineStr">
+      <c r="F110" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -6412,7 +6545,7 @@
         </is>
       </c>
       <c r="E111" s="2" t="n"/>
-      <c r="F111" s="3" t="inlineStr">
+      <c r="F111" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -6458,7 +6591,7 @@
         </is>
       </c>
       <c r="E112" s="2" t="n"/>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="F112" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6516,14 +6649,14 @@
         </is>
       </c>
       <c r="E113" s="2" t="n"/>
-      <c r="F113" s="3" t="inlineStr">
+      <c r="F113" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Evaluate/Statistics</t>
+          <t>Localization Statistics, per_region</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
@@ -6541,6 +6674,11 @@
       <c r="L113" s="4" t="n"/>
       <c r="M113" s="4" t="n"/>
       <c r="N113" s="2" t="inlineStr"/>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Localization Statistics is per_region now</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="2" t="n">
@@ -6562,14 +6700,14 @@
         </is>
       </c>
       <c r="E114" s="2" t="n"/>
-      <c r="F114" s="3" t="inlineStr">
+      <c r="F114" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>NPC Corners</t>
+          <t>Analysis/Measure/NPC Corners</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
@@ -6587,6 +6725,11 @@
       <c r="L114" s="4" t="n"/>
       <c r="M114" s="4" t="n"/>
       <c r="N114" s="2" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>moved to Analysis/Measure/NPC Corners (per_region)</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="42" customHeight="1">
       <c r="A115" s="2" t="n">
@@ -6608,7 +6751,7 @@
         </is>
       </c>
       <c r="E115" s="2" t="n"/>
-      <c r="F115" s="6" t="inlineStr">
+      <c r="F115" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6670,7 +6813,7 @@
         </is>
       </c>
       <c r="E116" s="2" t="n"/>
-      <c r="F116" s="4" t="inlineStr">
+      <c r="F116" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -6709,6 +6852,11 @@
       <c r="N116" s="2" t="inlineStr">
         <is>
           <t>E5 Circle / NPC geometry</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>build as a per_region Measure plugin</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6880,7 @@
         </is>
       </c>
       <c r="E117" s="2" t="n"/>
-      <c r="F117" s="6" t="inlineStr">
+      <c r="F117" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6771,6 +6919,11 @@
       <c r="N117" s="2" t="inlineStr">
         <is>
           <t>E3 Segmenter</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>as a Regions action, using E5 circle fit</t>
         </is>
       </c>
     </row>
@@ -6794,7 +6947,7 @@
         </is>
       </c>
       <c r="E118" s="2" t="n"/>
-      <c r="F118" s="6" t="inlineStr">
+      <c r="F118" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6833,6 +6986,11 @@
       <c r="N118" s="2" t="inlineStr">
         <is>
           <t>H LocMoFit</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>model fit = per_region Measure plugin; params become region values</t>
         </is>
       </c>
     </row>
@@ -6856,14 +7014,14 @@
         </is>
       </c>
       <c r="E119" s="2" t="n"/>
-      <c r="F119" s="4" t="inlineStr">
+      <c r="F119" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Line Profile is not a site evaluator</t>
+          <t>per_region framework done; Line Profile not per_region</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
@@ -6895,6 +7053,11 @@
       <c r="N119" s="2" t="inlineStr">
         <is>
           <t>E4 Evaluator = analysis</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>framework DONE (per_region replaces evaluators); Line Profile itself not per_region yet</t>
         </is>
       </c>
     </row>
@@ -6918,7 +7081,7 @@
         </is>
       </c>
       <c r="E120" s="2" t="n"/>
-      <c r="F120" s="6" t="inlineStr">
+      <c r="F120" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -6980,7 +7143,7 @@
         </is>
       </c>
       <c r="E121" s="2" t="n"/>
-      <c r="F121" s="6" t="inlineStr">
+      <c r="F121" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7015,6 +7178,11 @@
       <c r="N121" s="2" t="inlineStr">
         <is>
           <t>B2 Cluster</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>see #96: done by structure</t>
         </is>
       </c>
     </row>
@@ -7038,7 +7206,7 @@
         </is>
       </c>
       <c r="E122" s="2" t="n"/>
-      <c r="F122" s="6" t="inlineStr">
+      <c r="F122" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7073,6 +7241,11 @@
       <c r="N122" s="2" t="inlineStr">
         <is>
           <t>B4 Counting</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>with B4: per_region measure + Summarize</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7319,7 @@
         </is>
       </c>
       <c r="E124" s="2" t="n"/>
-      <c r="F124" s="4" t="inlineStr">
+      <c r="F124" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -7196,7 +7369,7 @@
         </is>
       </c>
       <c r="E125" s="2" t="n"/>
-      <c r="F125" s="6" t="inlineStr">
+      <c r="F125" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7254,14 +7427,14 @@
         </is>
       </c>
       <c r="E126" s="2" t="n"/>
-      <c r="F126" s="3" t="inlineStr">
+      <c r="F126" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>chains/batch, NPC chain</t>
+          <t>chains with blocks (per region)</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -7279,6 +7452,11 @@
       <c r="L126" s="4" t="n"/>
       <c r="M126" s="4" t="n"/>
       <c r="N126" s="2" t="inlineStr"/>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>blocks of a chain now</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="28" customHeight="1">
       <c r="A127" s="2" t="n">
@@ -7300,7 +7478,7 @@
         </is>
       </c>
       <c r="E127" s="2" t="n"/>
-      <c r="F127" s="3" t="inlineStr">
+      <c r="F127" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -7346,12 +7524,16 @@
         </is>
       </c>
       <c r="E128" s="2" t="n"/>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="G128" s="2" t="n"/>
+      <c r="F128" s="14" t="inlineStr">
+        <is>
+          <t>have</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Regions/Filter ROIs</t>
+        </is>
+      </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7380,7 +7562,12 @@
       <c r="M128" s="4" t="n"/>
       <c r="N128" s="2" t="inlineStr">
         <is>
-          <t>E1 ROI housekeeping</t>
+          <t>E1 done</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>DONE: Analysis/Regions/Filter ROIs</t>
         </is>
       </c>
     </row>
@@ -7404,12 +7591,16 @@
         </is>
       </c>
       <c r="E129" s="2" t="n"/>
-      <c r="F129" s="6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="G129" s="2" t="n"/>
+      <c r="F129" s="14" t="inlineStr">
+        <is>
+          <t>have</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>Regions/Sort ROIs</t>
+        </is>
+      </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
           <t>P2</t>
@@ -7438,7 +7629,12 @@
       </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
-          <t>E1 ROI housekeeping</t>
+          <t>E1 done</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>DONE: Analysis/Regions/Sort ROIs</t>
         </is>
       </c>
     </row>
@@ -7462,7 +7658,7 @@
         </is>
       </c>
       <c r="E130" s="2" t="n"/>
-      <c r="F130" s="6" t="inlineStr">
+      <c r="F130" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7493,6 +7689,11 @@
       <c r="N130" s="2" t="inlineStr">
         <is>
           <t>E1 ROI housekeeping</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>open; small Regions plugin or a Filter ROIs mode</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7717,7 @@
         </is>
       </c>
       <c r="E131" s="2" t="n"/>
-      <c r="F131" s="4" t="inlineStr">
+      <c r="F131" s="15" t="inlineStr">
         <is>
           <t>partly</t>
         </is>
@@ -7558,7 +7759,12 @@
       </c>
       <c r="N131" s="2" t="inlineStr">
         <is>
-          <t>E1 ROI housekeeping</t>
+          <t>A7 Export region table</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>still open: no CSV of the region table; now plan A7 (Summarize plugin over region_results)</t>
         </is>
       </c>
     </row>
@@ -7582,12 +7788,16 @@
         </is>
       </c>
       <c r="E132" s="2" t="n"/>
-      <c r="F132" s="6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="G132" s="2" t="n"/>
+      <c r="F132" s="14" t="inlineStr">
+        <is>
+          <t>have</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Regions/Regions to column</t>
+        </is>
+      </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
           <t>P2</t>
@@ -7620,7 +7830,12 @@
       </c>
       <c r="N132" s="2" t="inlineStr">
         <is>
-          <t>E1 ROI housekeeping</t>
+          <t>E1 done</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>DONE: Analysis/Regions/Regions to column (roi_id too), block write values</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7859,7 @@
         </is>
       </c>
       <c r="E133" s="2" t="n"/>
-      <c r="F133" s="6" t="inlineStr">
+      <c r="F133" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7679,6 +7894,11 @@
       <c r="N133" s="2" t="inlineStr">
         <is>
           <t>E6 Site figures</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>open; Summarize-style plugin reading ROI order and annotations</t>
         </is>
       </c>
     </row>
@@ -7702,7 +7922,7 @@
         </is>
       </c>
       <c r="E134" s="2" t="n"/>
-      <c r="F134" s="6" t="inlineStr">
+      <c r="F134" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7760,7 +7980,7 @@
         </is>
       </c>
       <c r="E135" s="2" t="n"/>
-      <c r="F135" s="6" t="inlineStr">
+      <c r="F135" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7799,6 +8019,11 @@
       <c r="N135" s="2" t="inlineStr">
         <is>
           <t>E7 Average sites</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>open; needs named lines per ROI (E2)</t>
         </is>
       </c>
     </row>
@@ -7822,7 +8047,7 @@
         </is>
       </c>
       <c r="E136" s="2" t="n"/>
-      <c r="F136" s="6" t="inlineStr">
+      <c r="F136" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7876,7 +8101,7 @@
         </is>
       </c>
       <c r="E137" s="2" t="n"/>
-      <c r="F137" s="6" t="inlineStr">
+      <c r="F137" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7922,7 +8147,7 @@
         </is>
       </c>
       <c r="E138" s="2" t="n"/>
-      <c r="F138" s="6" t="inlineStr">
+      <c r="F138" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -7968,7 +8193,7 @@
           <t>fit geometric/image models to each site's localizations, model selection; drives averaging</t>
         </is>
       </c>
-      <c r="F139" s="6" t="inlineStr">
+      <c r="F139" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8007,6 +8232,11 @@
       <c r="N139" s="2" t="inlineStr">
         <is>
           <t>H LocMoFit</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>model fit = per_region Measure plugin; params become region values</t>
         </is>
       </c>
     </row>
@@ -8030,7 +8260,7 @@
           <t>sliding-window reconstruction movie (live cell)</t>
         </is>
       </c>
-      <c r="F140" s="6" t="inlineStr">
+      <c r="F140" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8092,7 +8322,7 @@
           <t>raw frames beside a building-up SR image</t>
         </is>
       </c>
-      <c r="F141" s="6" t="inlineStr">
+      <c r="F141" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8150,7 +8380,7 @@
         </is>
       </c>
       <c r="E142" s="2" t="n"/>
-      <c r="F142" s="6" t="inlineStr">
+      <c r="F142" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8204,7 +8434,7 @@
         </is>
       </c>
       <c r="E143" s="2" t="n"/>
-      <c r="F143" s="3" t="inlineStr">
+      <c r="F143" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -8246,7 +8476,7 @@
         </is>
       </c>
       <c r="E144" s="2" t="n"/>
-      <c r="F144" s="3" t="inlineStr">
+      <c r="F144" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -8288,7 +8518,7 @@
         </is>
       </c>
       <c r="E145" s="2" t="n"/>
-      <c r="F145" s="3" t="inlineStr">
+      <c r="F145" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -8326,7 +8556,7 @@
         </is>
       </c>
       <c r="E146" s="2" t="n"/>
-      <c r="F146" s="3" t="inlineStr">
+      <c r="F146" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -8368,7 +8598,7 @@
         </is>
       </c>
       <c r="E147" s="2" t="n"/>
-      <c r="F147" s="3" t="inlineStr">
+      <c r="F147" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -8410,7 +8640,7 @@
         </is>
       </c>
       <c r="E148" s="2" t="n"/>
-      <c r="F148" s="3" t="inlineStr">
+      <c r="F148" s="14" t="inlineStr">
         <is>
           <t>have</t>
         </is>
@@ -8456,7 +8686,7 @@
           <t>CME / yeast</t>
         </is>
       </c>
-      <c r="F149" s="6" t="inlineStr">
+      <c r="F149" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8498,7 +8728,7 @@
           <t>Fibrils / BALM</t>
         </is>
       </c>
-      <c r="F150" s="6" t="inlineStr">
+      <c r="F150" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8540,7 +8770,7 @@
           <t>Platelets, polarization, misc. projects</t>
         </is>
       </c>
-      <c r="F151" s="6" t="inlineStr">
+      <c r="F151" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8582,7 +8812,7 @@
           <t>Kinetochore</t>
         </is>
       </c>
-      <c r="F152" s="6" t="inlineStr">
+      <c r="F152" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8624,7 +8854,7 @@
           <t>MINFLUX analysis</t>
         </is>
       </c>
-      <c r="F153" s="6" t="inlineStr">
+      <c r="F153" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8678,7 +8908,7 @@
           <t>Model-fit summaries</t>
         </is>
       </c>
-      <c r="F154" s="6" t="inlineStr">
+      <c r="F154" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8720,7 +8950,7 @@
           <t>Duplicates / dead</t>
         </is>
       </c>
-      <c r="F155" s="6" t="inlineStr">
+      <c r="F155" s="16" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
@@ -8742,13 +8972,88 @@
       <c r="M155" s="4" t="n"/>
       <c r="N155" s="2" t="inlineStr"/>
     </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t>12. ROI manager</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Annotate</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>SEAnnotation (GUI panel)</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>label lists per ROI, keyboard navigation, comment, two drawn lines with angle/length</t>
+        </is>
+      </c>
+      <c r="F156" s="15" t="inlineStr">
+        <is>
+          <t>partly</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>gui/roi_annotate.py: keyword lists, keys 1-9, Tab, Up/Down, Space=use, comment; one direction line only</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>add several named lines per ROI (angle, length as values)</t>
+        </is>
+      </c>
+      <c r="K156" s="4" t="inlineStr">
+        <is>
+          <t>work on</t>
+        </is>
+      </c>
+      <c r="L156" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="M156" s="4" t="inlineStr">
+        <is>
+          <t>(added from your message: annotate ROI plugin incl. several lines)</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr">
+        <is>
+          <t>E2 Annotate ROIs</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>mostly DONE; missing: several named lines per ROI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N155"/>
+  <autoFilter ref="A1:O156"/>
   <dataValidations count="2">
-    <dataValidation sqref="K2:K155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"work on,change,later,skip,done"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P1,P2,P3,skip"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Porting plan: segmentation (Find clusters, Segment regions) kept apart from local density, shuffle colours for any id
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4rjWo2i91xceLvMFCkyKa
</commit_message>
<xml_diff>
--- a/docs/smap_porting/SMAP_porting_list.xlsx
+++ b/docs/smap_porting/SMAP_porting_list.xlsx
@@ -4320,6 +4320,11 @@
           <t>B1 Neighbourhood</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>decided: Neighbourhood plugin (local density, field statistics around each loc); writes columns, no segmentation</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="56" customHeight="1">
       <c r="A72" s="2" t="n">
@@ -5424,12 +5429,12 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>B2 Cluster</t>
+          <t>B2 Find clusters</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>DONE: Analysis/Regions/Find/DBSCAN (cluster_id, n_in_cluster)</t>
+          <t>DBSCAN done (Regions/Find/DBSCAN); decided: fold into one "Find clusters" plugin with algorithm choice (DBSCAN, HDBSCAN, Voronoi, ...)</t>
         </is>
       </c>
     </row>
@@ -5549,12 +5554,12 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>B1/B2 Neighbourhood + Cluster</t>
+          <t>B1 Neighbourhood + B2 Find clusters</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>open; as another Regions/Find plugin (B2) + density in Neighbourhood (B1)</t>
+          <t>decided: Voronoi density -&gt; Neighbourhood (B1); Voronoi clustering -&gt; an algorithm of Find clusters (B2)</t>
         </is>
       </c>
     </row>
@@ -5619,6 +5624,11 @@
           <t>B1 Neighbourhood</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>decided: part of Neighbourhood (B1)</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="70" customHeight="1">
       <c r="A96" s="2" t="n">
@@ -5678,12 +5688,12 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>B2 Cluster</t>
+          <t>B2s Shuffle colours</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>open; suggest a render/LUT option for any id column, not cluster-only</t>
+          <t>decided: separate small plugin for ANY integer column (cluster_id, roi_id, tid, frame...)</t>
         </is>
       </c>
     </row>
@@ -6206,12 +6216,12 @@
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>E3 Segmenter</t>
+          <t>B2/E3 Segment regions</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>finders and clusterers are one kind now (Regions/Find); presets still open</t>
+          <t>decided: fold Find/NPC into one "Segment regions" plugin with presets (NPC, Density Peaks, templates)</t>
         </is>
       </c>
     </row>
@@ -6269,12 +6279,12 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>E3 Segmenter</t>
+          <t>B2/E3 Segment regions</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Regions/Find/Density Peaks; presets / one-vs-many plugins still open</t>
+          <t>decided: Density Peaks -&gt; preset of "Segment regions"</t>
         </is>
       </c>
     </row>
@@ -6521,7 +6531,12 @@
       </c>
       <c r="N110" s="2" t="inlineStr">
         <is>
-          <t>E3 Segmenter</t>
+          <t>B2/E3 Segment regions</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>decided: a preset of "Segment regions"</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6640,12 @@
       </c>
       <c r="N112" s="2" t="inlineStr">
         <is>
-          <t>E3 Segmenter</t>
+          <t>B2/E3 Segment regions</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>decided: CME etc. as presets/templates of "Segment regions"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Porting plan: an implementation plan in waves, settings of unselected algorithms hidden
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4rjWo2i91xceLvMFCkyKa
</commit_message>
<xml_diff>
--- a/docs/smap_porting/SMAP_porting_list.xlsx
+++ b/docs/smap_porting/SMAP_porting_list.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Port list'!$A$1:$O$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Port list'!$A$1:$P$156</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O156"/>
+  <dimension ref="A1:P156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="7.6640625" customWidth="1" min="3" max="3"/>
@@ -549,6 +549,7 @@
     <col width="21.83203125" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -627,6 +628,11 @@
           <t>Update 2026-10-14</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Plan step</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -673,6 +679,7 @@
       <c r="L2" s="4" t="n"/>
       <c r="M2" s="4" t="n"/>
       <c r="N2" s="2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -719,6 +726,7 @@
       <c r="L3" s="4" t="n"/>
       <c r="M3" s="4" t="n"/>
       <c r="N3" s="2" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -769,6 +777,7 @@
       <c r="L4" s="4" t="n"/>
       <c r="M4" s="4" t="n"/>
       <c r="N4" s="2" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" ht="56" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -819,6 +828,7 @@
       <c r="L5" s="4" t="n"/>
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="2" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -857,6 +867,7 @@
       <c r="L6" s="4" t="n"/>
       <c r="M6" s="4" t="n"/>
       <c r="N6" s="2" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -915,6 +926,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="56" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -973,6 +985,11 @@
           <t>A3 Fit region</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1019,6 +1036,7 @@
       <c r="L9" s="4" t="n"/>
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="2" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -1069,6 +1087,7 @@
       <c r="L10" s="4" t="n"/>
       <c r="M10" s="4" t="n"/>
       <c r="N10" s="2" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -1131,6 +1150,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -1193,6 +1213,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -1239,6 +1260,7 @@
       <c r="L13" s="4" t="n"/>
       <c r="M13" s="4" t="n"/>
       <c r="N13" s="2" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -1293,6 +1315,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -1343,6 +1366,7 @@
       <c r="L15" s="4" t="n"/>
       <c r="M15" s="4" t="n"/>
       <c r="N15" s="2" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -1405,6 +1429,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1451,6 +1476,7 @@
       <c r="L17" s="4" t="n"/>
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="2" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1501,6 +1527,7 @@
       <c r="L18" s="4" t="n"/>
       <c r="M18" s="4" t="n"/>
       <c r="N18" s="2" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -1547,6 +1574,7 @@
       <c r="L19" s="4" t="n"/>
       <c r="M19" s="4" t="n"/>
       <c r="N19" s="2" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1597,6 +1625,7 @@
       <c r="L20" s="4" t="n"/>
       <c r="M20" s="4" t="n"/>
       <c r="N20" s="2" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1643,6 +1672,7 @@
       <c r="L21" s="4" t="n"/>
       <c r="M21" s="4" t="n"/>
       <c r="N21" s="2" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1685,6 +1715,7 @@
       <c r="L22" s="4" t="n"/>
       <c r="M22" s="4" t="n"/>
       <c r="N22" s="2" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -1751,6 +1782,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -1797,6 +1829,7 @@
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="2" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25" ht="56" customHeight="1">
       <c r="A25" s="2" t="n">
@@ -1855,6 +1888,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -1901,6 +1935,7 @@
       <c r="L26" s="4" t="n"/>
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="2" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" ht="84" customHeight="1">
       <c r="A27" s="2" t="n">
@@ -1963,6 +1998,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28" ht="56" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -2025,6 +2061,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="2" t="n">
@@ -2071,6 +2108,7 @@
       <c r="L29" s="4" t="n"/>
       <c r="M29" s="4" t="n"/>
       <c r="N29" s="2" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30" ht="56" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -2129,6 +2167,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="2" t="n">
@@ -2175,6 +2214,7 @@
       <c r="L31" s="4" t="n"/>
       <c r="M31" s="4" t="n"/>
       <c r="N31" s="2" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -2217,6 +2257,7 @@
       <c r="L32" s="4" t="n"/>
       <c r="M32" s="4" t="n"/>
       <c r="N32" s="2" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="2" t="n">
@@ -2263,6 +2304,7 @@
       <c r="L33" s="4" t="n"/>
       <c r="M33" s="4" t="n"/>
       <c r="N33" s="2" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="2" t="n">
@@ -2309,6 +2351,7 @@
       <c r="L34" s="4" t="n"/>
       <c r="M34" s="4" t="n"/>
       <c r="N34" s="2" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35" ht="70" customHeight="1">
       <c r="A35" s="2" t="n">
@@ -2367,6 +2410,11 @@
           <t>D2 Fiducial drift</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>wave 5 (D2)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="42" customHeight="1">
       <c r="A36" s="2" t="n">
@@ -2425,6 +2473,11 @@
           <t>D1 Apply drift</t>
         </is>
       </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>wave 5 (D1)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="2" t="n">
@@ -2483,6 +2536,7 @@
           <t>D later</t>
         </is>
       </c>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -2529,6 +2583,7 @@
       <c r="L38" s="4" t="n"/>
       <c r="M38" s="4" t="n"/>
       <c r="N38" s="2" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39" ht="70" customHeight="1">
       <c r="A39" s="2" t="n">
@@ -2587,6 +2642,11 @@
           <t>D3 COMET time-dep. transform</t>
         </is>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>wave 5 (D3)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="42" customHeight="1">
       <c r="A40" s="2" t="n">
@@ -2649,6 +2709,7 @@
           <t>C later</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41" ht="98" customHeight="1">
       <c r="A41" s="2" t="n">
@@ -2715,6 +2776,11 @@
           <t>C1 Transform</t>
         </is>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>wave 5 (C1)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="196" customHeight="1">
       <c r="A42" s="2" t="n">
@@ -2777,6 +2843,11 @@
           <t>C2/C3 Register layers, alignment diagnostic</t>
         </is>
       </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>wave 5 (C2/C3)</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="2" t="n">
@@ -2835,6 +2906,11 @@
           <t>C3 Alignment diagnostic</t>
         </is>
       </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>wave 5 (C3)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="56" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -2877,6 +2953,7 @@
       <c r="L44" s="4" t="n"/>
       <c r="M44" s="4" t="n"/>
       <c r="N44" s="2" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45" ht="42" customHeight="1">
       <c r="A45" s="2" t="n">
@@ -2935,6 +3012,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46" ht="42" customHeight="1">
       <c r="A46" s="2" t="n">
@@ -2981,6 +3059,7 @@
       <c r="L46" s="4" t="n"/>
       <c r="M46" s="4" t="n"/>
       <c r="N46" s="2" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47" ht="126" customHeight="1">
       <c r="A47" s="2" t="n">
@@ -3043,6 +3122,7 @@
           <t>C later</t>
         </is>
       </c>
+      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48" ht="56" customHeight="1">
       <c r="A48" s="2" t="n">
@@ -3103,6 +3183,11 @@
       <c r="N48" s="2" t="inlineStr">
         <is>
           <t>C4 AssignColors &gt;2</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>wave 5 (C4)</t>
         </is>
       </c>
     </row>
@@ -3152,6 +3237,7 @@
           <t>one loader now (File/Load/Auto) with a format choice</t>
         </is>
       </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -3198,6 +3284,7 @@
       <c r="L50" s="4" t="n"/>
       <c r="M50" s="4" t="n"/>
       <c r="N50" s="2" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="2" t="n">
@@ -3244,6 +3331,7 @@
       <c r="L51" s="4" t="n"/>
       <c r="M51" s="4" t="n"/>
       <c r="N51" s="2" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="2" t="n">
@@ -3307,6 +3395,11 @@
           <t>smaller now: a Reader in io/formats.py, not a plugin</t>
         </is>
       </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="2" t="n">
@@ -3370,6 +3463,11 @@
           <t>smaller now: a Reader in io/formats.py, not a plugin</t>
         </is>
       </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="2" t="n">
@@ -3424,6 +3522,11 @@
           <t>A1 Export</t>
         </is>
       </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="112" customHeight="1">
       <c r="A55" s="2" t="n">
@@ -3482,6 +3585,11 @@
           <t>A1 Export</t>
         </is>
       </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="2" t="n">
@@ -3536,6 +3644,11 @@
           <t>A1 Export</t>
         </is>
       </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>2 (optional format)</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="2" t="n">
@@ -3582,6 +3695,7 @@
       <c r="L57" s="4" t="n"/>
       <c r="M57" s="4" t="n"/>
       <c r="N57" s="2" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
     </row>
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="2" t="n">
@@ -3632,6 +3746,7 @@
       <c r="L58" s="4" t="n"/>
       <c r="M58" s="4" t="n"/>
       <c r="N58" s="2" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3674,6 +3789,7 @@
       <c r="L59" s="4" t="n"/>
       <c r="M59" s="4" t="n"/>
       <c r="N59" s="2" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="2" t="n">
@@ -3720,6 +3836,7 @@
       <c r="L60" s="4" t="n"/>
       <c r="M60" s="4" t="n"/>
       <c r="N60" s="2" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3762,6 +3879,7 @@
       <c r="L61" s="4" t="n"/>
       <c r="M61" s="4" t="n"/>
       <c r="N61" s="2" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
     </row>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="2" t="n">
@@ -3808,6 +3926,7 @@
       <c r="L62" s="4" t="n"/>
       <c r="M62" s="4" t="n"/>
       <c r="N62" s="2" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63" ht="84" customHeight="1">
       <c r="A63" s="2" t="n">
@@ -3850,6 +3969,7 @@
       <c r="L63" s="4" t="n"/>
       <c r="M63" s="4" t="n"/>
       <c r="N63" s="2" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
     </row>
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="2" t="n">
@@ -3901,6 +4021,7 @@
           <t>moved to Analysis/Process/Layers</t>
         </is>
       </c>
+      <c r="P64" t="inlineStr"/>
     </row>
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="2" t="n">
@@ -3947,6 +4068,7 @@
       <c r="L65" s="4" t="n"/>
       <c r="M65" s="4" t="n"/>
       <c r="N65" s="2" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
     </row>
     <row r="66" ht="56" customHeight="1">
       <c r="A66" s="2" t="n">
@@ -4013,6 +4135,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P66" t="inlineStr"/>
     </row>
     <row r="67" ht="56" customHeight="1">
       <c r="A67" s="2" t="n">
@@ -4075,6 +4198,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P67" t="inlineStr"/>
     </row>
     <row r="68" ht="56" customHeight="1">
       <c r="A68" s="2" t="n">
@@ -4142,6 +4266,7 @@
           <t>measuring per id: done (block over any id column); collapsing a region into one row still open, see plan J</t>
         </is>
       </c>
+      <c r="P68" t="inlineStr"/>
     </row>
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="2" t="n">
@@ -4196,6 +4321,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P69" t="inlineStr"/>
     </row>
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="2" t="n">
@@ -4258,6 +4384,11 @@
           <t>C1 Transform</t>
         </is>
       </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>wave 5 (C1)</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="56" customHeight="1">
       <c r="A71" s="2" t="n">
@@ -4325,6 +4456,11 @@
           <t>decided: Neighbourhood plugin (local density, field statistics around each loc); writes columns, no segmentation</t>
         </is>
       </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="56" customHeight="1">
       <c r="A72" s="2" t="n">
@@ -4375,6 +4511,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P72" t="inlineStr"/>
     </row>
     <row r="73" ht="84" customHeight="1">
       <c r="A73" s="2" t="n">
@@ -4417,6 +4554,7 @@
       <c r="L73" s="4" t="n"/>
       <c r="M73" s="4" t="n"/>
       <c r="N73" s="2" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="2" t="n">
@@ -4463,6 +4601,7 @@
       <c r="L74" s="4" t="n"/>
       <c r="M74" s="4" t="n"/>
       <c r="N74" s="2" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75" ht="98" customHeight="1">
       <c r="A75" s="2" t="n">
@@ -4525,6 +4664,11 @@
           <t>C1 Transform</t>
         </is>
       </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>wave 5 (C1)</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="42" customHeight="1">
       <c r="A76" s="2" t="n">
@@ -4571,6 +4715,7 @@
       <c r="L76" s="4" t="n"/>
       <c r="M76" s="4" t="n"/>
       <c r="N76" s="2" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
     </row>
     <row r="77" ht="56" customHeight="1">
       <c r="A77" s="2" t="n">
@@ -4633,6 +4778,11 @@
           <t>I Rendering/movies</t>
         </is>
       </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>wave 5 (I)</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="2" t="n">
@@ -4691,6 +4841,11 @@
           <t>I Rendering/movies</t>
         </is>
       </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>wave 5 (I)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="42" customHeight="1">
       <c r="A79" s="2" t="n">
@@ -4737,6 +4892,7 @@
       <c r="L79" s="4" t="n"/>
       <c r="M79" s="4" t="n"/>
       <c r="N79" s="2" t="inlineStr"/>
+      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="2" t="n">
@@ -4783,6 +4939,7 @@
       <c r="L80" s="4" t="n"/>
       <c r="M80" s="4" t="n"/>
       <c r="N80" s="2" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
     </row>
     <row r="81" ht="42" customHeight="1">
       <c r="A81" s="2" t="n">
@@ -4833,6 +4990,7 @@
       <c r="L81" s="4" t="n"/>
       <c r="M81" s="4" t="n"/>
       <c r="N81" s="2" t="inlineStr"/>
+      <c r="P81" t="inlineStr"/>
     </row>
     <row r="82" ht="98" customHeight="1">
       <c r="A82" s="2" t="n">
@@ -4887,6 +5045,7 @@
           <t>I Rendering/movies</t>
         </is>
       </c>
+      <c r="P82" t="inlineStr"/>
     </row>
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="2" t="n">
@@ -4933,6 +5092,7 @@
       <c r="L83" s="4" t="n"/>
       <c r="M83" s="4" t="n"/>
       <c r="N83" s="2" t="inlineStr"/>
+      <c r="P83" t="inlineStr"/>
     </row>
     <row r="84" ht="42" customHeight="1">
       <c r="A84" s="2" t="n">
@@ -4979,6 +5139,7 @@
       <c r="L84" s="4" t="n"/>
       <c r="M84" s="4" t="n"/>
       <c r="N84" s="2" t="inlineStr"/>
+      <c r="P84" t="inlineStr"/>
     </row>
     <row r="85" ht="42" customHeight="1">
       <c r="A85" s="2" t="n">
@@ -5029,6 +5190,7 @@
       <c r="L85" s="4" t="n"/>
       <c r="M85" s="4" t="n"/>
       <c r="N85" s="2" t="inlineStr"/>
+      <c r="P85" t="inlineStr"/>
     </row>
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="2" t="n">
@@ -5075,6 +5237,7 @@
       <c r="L86" s="4" t="n"/>
       <c r="M86" s="4" t="n"/>
       <c r="N86" s="2" t="inlineStr"/>
+      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87" ht="56" customHeight="1">
       <c r="A87" s="2" t="n">
@@ -5142,6 +5305,11 @@
           <t>Regions/Summarize/Histograms = over regions; histogram of localizations still open (A4); make it per_region too</t>
         </is>
       </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="56" customHeight="1">
       <c r="A88" s="2" t="n">
@@ -5208,6 +5376,11 @@
           <t>A5 Time course</t>
         </is>
       </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="28" customHeight="1">
       <c r="A89" s="2" t="n">
@@ -5266,6 +5439,11 @@
           <t>A6 Vibrations</t>
         </is>
       </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>wave 5 (A6)</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="42" customHeight="1">
       <c r="A90" s="2" t="n">
@@ -5312,6 +5490,7 @@
       <c r="L90" s="4" t="n"/>
       <c r="M90" s="4" t="n"/>
       <c r="N90" s="2" t="inlineStr"/>
+      <c r="P90" t="inlineStr"/>
     </row>
     <row r="91" ht="98" customHeight="1">
       <c r="A91" s="2" t="n">
@@ -5366,6 +5545,11 @@
           <t>B3 Spatial statistics</t>
         </is>
       </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="112" customHeight="1">
       <c r="A92" s="2" t="n">
@@ -5437,6 +5621,11 @@
           <t>DBSCAN done (Regions/Find/DBSCAN); decided: fold into one "Find clusters" plugin with algorithm choice (DBSCAN, HDBSCAN, Voronoi, ...)</t>
         </is>
       </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="98" customHeight="1">
       <c r="A93" s="2" t="n">
@@ -5499,6 +5688,11 @@
           <t>B3 Spatial statistics</t>
         </is>
       </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="42" customHeight="1">
       <c r="A94" s="2" t="n">
@@ -5562,6 +5756,11 @@
           <t>decided: Voronoi density -&gt; Neighbourhood (B1); Voronoi clustering -&gt; an algorithm of Find clusters (B2)</t>
         </is>
       </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>9 + 10</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="84" customHeight="1">
       <c r="A95" s="2" t="n">
@@ -5629,6 +5828,11 @@
           <t>decided: part of Neighbourhood (B1)</t>
         </is>
       </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="70" customHeight="1">
       <c r="A96" s="2" t="n">
@@ -5696,6 +5900,11 @@
           <t>decided: separate small plugin for ANY integer column (cluster_id, roi_id, tid, frame...)</t>
         </is>
       </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="42" customHeight="1">
       <c r="A97" s="2" t="n">
@@ -5767,6 +5976,11 @@
           <t>DONE by structure: block over cluster_id (nested in ROIs) with any per_region plugin; a cluster-shape measurement still open (B2b)</t>
         </is>
       </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -5809,6 +6023,7 @@
       <c r="L98" s="4" t="n"/>
       <c r="M98" s="4" t="n"/>
       <c r="N98" s="2" t="inlineStr"/>
+      <c r="P98" t="inlineStr"/>
     </row>
     <row r="99" ht="112" customHeight="1">
       <c r="A99" s="2" t="n">
@@ -5876,6 +6091,11 @@
           <t>clear path now: per_region measure + Summarize fit (like NPC Corners + labelling efficiency)</t>
         </is>
       </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="70" customHeight="1">
       <c r="A100" s="2" t="n">
@@ -5918,6 +6138,7 @@
       <c r="L100" s="4" t="n"/>
       <c r="M100" s="4" t="n"/>
       <c r="N100" s="2" t="inlineStr"/>
+      <c r="P100" t="inlineStr"/>
     </row>
     <row r="101" ht="126" customHeight="1">
       <c r="A101" s="2" t="n">
@@ -5985,6 +6206,11 @@
           <t>tracks as an id column (track_id) -&gt; per_region plugins run per track for free</t>
         </is>
       </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="56" customHeight="1">
       <c r="A102" s="2" t="n">
@@ -6052,6 +6278,11 @@
           <t>analyses as per_region measures + summaries over tracks</t>
         </is>
       </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -6098,6 +6329,7 @@
       <c r="L103" s="4" t="n"/>
       <c r="M103" s="4" t="n"/>
       <c r="N103" s="2" t="inlineStr"/>
+      <c r="P103" t="inlineStr"/>
     </row>
     <row r="104" ht="126" customHeight="1">
       <c r="A104" s="2" t="n">
@@ -6161,6 +6393,11 @@
           <t>tid is already an id column -&gt; per-trace via regions</t>
         </is>
       </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>wave 5 (G)</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="70" customHeight="1">
       <c r="A105" s="2" t="n">
@@ -6224,6 +6461,11 @@
           <t>decided: fold Find/NPC into one "Segment regions" plugin with presets (NPC, Density Peaks, templates)</t>
         </is>
       </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="42" customHeight="1">
       <c r="A106" s="2" t="n">
@@ -6287,6 +6529,11 @@
           <t>decided: Density Peaks -&gt; preset of "Segment regions"</t>
         </is>
       </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="2" t="n">
@@ -6350,6 +6597,11 @@
           <t>open; could be a Filter ROIs condition on position</t>
         </is>
       </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="2" t="n">
@@ -6411,6 +6663,11 @@
       <c r="O108" t="inlineStr">
         <is>
           <t>open; suggest a third region choice of Remove Localizations; for clusters a filter cluster_id&gt;0 does it</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -6472,6 +6729,7 @@
           <t>mostly there: Column to ROIs on filenumber</t>
         </is>
       </c>
+      <c r="P109" t="inlineStr"/>
     </row>
     <row r="110" ht="56" customHeight="1">
       <c r="A110" s="2" t="n">
@@ -6539,6 +6797,11 @@
           <t>decided: a preset of "Segment regions"</t>
         </is>
       </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>11 (later preset)</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="2" t="n">
@@ -6585,6 +6848,7 @@
       <c r="L111" s="4" t="n"/>
       <c r="M111" s="4" t="n"/>
       <c r="N111" s="2" t="inlineStr"/>
+      <c r="P111" t="inlineStr"/>
     </row>
     <row r="112" ht="98" customHeight="1">
       <c r="A112" s="2" t="n">
@@ -6646,6 +6910,11 @@
       <c r="O112" t="inlineStr">
         <is>
           <t>decided: CME etc. as presets/templates of "Segment regions"</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>11 (later presets)</t>
         </is>
       </c>
     </row>
@@ -6699,6 +6968,7 @@
           <t>Localization Statistics is per_region now</t>
         </is>
       </c>
+      <c r="P113" t="inlineStr"/>
     </row>
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="2" t="n">
@@ -6750,6 +7020,7 @@
           <t>moved to Analysis/Measure/NPC Corners (per_region)</t>
         </is>
       </c>
+      <c r="P114" t="inlineStr"/>
     </row>
     <row r="115" ht="42" customHeight="1">
       <c r="A115" s="2" t="n">
@@ -6812,6 +7083,11 @@
           <t>E5 Circle / NPC geometry</t>
         </is>
       </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>wave 5 (H/E5)</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="42" customHeight="1">
       <c r="A116" s="2" t="n">
@@ -6879,6 +7155,11 @@
           <t>build as a per_region Measure plugin</t>
         </is>
       </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="56" customHeight="1">
       <c r="A117" s="2" t="n">
@@ -6946,6 +7227,11 @@
           <t>as a Regions action, using E5 circle fit</t>
         </is>
       </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="70" customHeight="1">
       <c r="A118" s="2" t="n">
@@ -7013,6 +7299,11 @@
           <t>model fit = per_region Measure plugin; params become region values</t>
         </is>
       </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>wave 5 (H)</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="84" customHeight="1">
       <c r="A119" s="2" t="n">
@@ -7080,6 +7371,11 @@
           <t>framework DONE (per_region replaces evaluators); Line Profile itself not per_region yet</t>
         </is>
       </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="112" customHeight="1">
       <c r="A120" s="2" t="n">
@@ -7142,6 +7438,11 @@
           <t>B3 + C2</t>
         </is>
       </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>17 (+ C2)</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="28" customHeight="1">
       <c r="A121" s="2" t="n">
@@ -7205,6 +7506,11 @@
           <t>see #96: done by structure</t>
         </is>
       </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="28" customHeight="1">
       <c r="A122" s="2" t="n">
@@ -7268,6 +7574,11 @@
           <t>with B4: per_region measure + Summarize</t>
         </is>
       </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="28" customHeight="1">
       <c r="A123" s="2" t="n">
@@ -7318,6 +7629,7 @@
       <c r="L123" s="4" t="n"/>
       <c r="M123" s="4" t="n"/>
       <c r="N123" s="2" t="inlineStr"/>
+      <c r="P123" t="inlineStr"/>
     </row>
     <row r="124" ht="42" customHeight="1">
       <c r="A124" s="2" t="n">
@@ -7368,6 +7680,7 @@
       <c r="L124" s="4" t="n"/>
       <c r="M124" s="4" t="n"/>
       <c r="N124" s="2" t="inlineStr"/>
+      <c r="P124" t="inlineStr"/>
     </row>
     <row r="125" ht="140" customHeight="1">
       <c r="A125" s="2" t="n">
@@ -7426,6 +7739,7 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="P125" t="inlineStr"/>
     </row>
     <row r="126" ht="28" customHeight="1">
       <c r="A126" s="2" t="n">
@@ -7477,6 +7791,7 @@
           <t>blocks of a chain now</t>
         </is>
       </c>
+      <c r="P126" t="inlineStr"/>
     </row>
     <row r="127" ht="28" customHeight="1">
       <c r="A127" s="2" t="n">
@@ -7523,6 +7838,7 @@
       <c r="L127" s="4" t="n"/>
       <c r="M127" s="4" t="n"/>
       <c r="N127" s="2" t="inlineStr"/>
+      <c r="P127" t="inlineStr"/>
     </row>
     <row r="128" ht="42" customHeight="1">
       <c r="A128" s="2" t="n">
@@ -7590,6 +7906,7 @@
           <t>DONE: Analysis/Regions/Filter ROIs</t>
         </is>
       </c>
+      <c r="P128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -7657,6 +7974,7 @@
           <t>DONE: Analysis/Regions/Sort ROIs</t>
         </is>
       </c>
+      <c r="P129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -7716,6 +8034,11 @@
           <t>open; small Regions plugin or a Filter ROIs mode</t>
         </is>
       </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="70" customHeight="1">
       <c r="A131" s="2" t="n">
@@ -7787,6 +8110,11 @@
           <t>still open: no CSV of the region table; now plan A7 (Summarize plugin over region_results)</t>
         </is>
       </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="56" customHeight="1">
       <c r="A132" s="2" t="n">
@@ -7858,6 +8186,7 @@
           <t>DONE: Analysis/Regions/Regions to column (roi_id too), block write values</t>
         </is>
       </c>
+      <c r="P132" t="inlineStr"/>
     </row>
     <row r="133" ht="56" customHeight="1">
       <c r="A133" s="2" t="n">
@@ -7921,6 +8250,11 @@
           <t>open; Summarize-style plugin reading ROI order and annotations</t>
         </is>
       </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>wave 5 (E6)</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="70" customHeight="1">
       <c r="A134" s="2" t="n">
@@ -7979,6 +8313,11 @@
           <t>E6 Site figures</t>
         </is>
       </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>wave 5 (E6)</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="98" customHeight="1">
       <c r="A135" s="2" t="n">
@@ -8046,6 +8385,11 @@
           <t>open; needs named lines per ROI (E2)</t>
         </is>
       </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -8100,6 +8444,7 @@
           <t>E1 ROI housekeeping</t>
         </is>
       </c>
+      <c r="P136" t="inlineStr"/>
     </row>
     <row r="137" ht="28" customHeight="1">
       <c r="A137" s="2" t="n">
@@ -8146,6 +8491,7 @@
       <c r="L137" s="4" t="n"/>
       <c r="M137" s="4" t="n"/>
       <c r="N137" s="2" t="inlineStr"/>
+      <c r="P137" t="inlineStr"/>
     </row>
     <row r="138" ht="266" customHeight="1">
       <c r="A138" s="2" t="n">
@@ -8192,6 +8538,7 @@
       <c r="L138" s="4" t="n"/>
       <c r="M138" s="4" t="n"/>
       <c r="N138" s="2" t="inlineStr"/>
+      <c r="P138" t="inlineStr"/>
     </row>
     <row r="139" ht="210" customHeight="1">
       <c r="A139" s="2" t="n">
@@ -8259,6 +8606,11 @@
           <t>model fit = per_region Measure plugin; params become region values</t>
         </is>
       </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>wave 5 (H)</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="56" customHeight="1">
       <c r="A140" s="2" t="n">
@@ -8321,6 +8673,11 @@
           <t>I Rendering/movies</t>
         </is>
       </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>wave 5 (I)</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="42" customHeight="1">
       <c r="A141" s="2" t="n">
@@ -8383,6 +8740,11 @@
           <t>I Rendering/movies</t>
         </is>
       </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>wave 5 (I)</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="42" customHeight="1">
       <c r="A142" s="2" t="n">
@@ -8437,6 +8799,11 @@
           <t>F SPT</t>
         </is>
       </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -8479,6 +8846,7 @@
       <c r="L143" s="4" t="n"/>
       <c r="M143" s="4" t="n"/>
       <c r="N143" s="2" t="inlineStr"/>
+      <c r="P143" t="inlineStr"/>
     </row>
     <row r="144" ht="42" customHeight="1">
       <c r="A144" s="2" t="n">
@@ -8521,6 +8889,7 @@
       <c r="L144" s="4" t="n"/>
       <c r="M144" s="4" t="n"/>
       <c r="N144" s="2" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
@@ -8559,6 +8928,7 @@
       <c r="L145" s="4" t="n"/>
       <c r="M145" s="4" t="n"/>
       <c r="N145" s="2" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
     </row>
     <row r="146" ht="28" customHeight="1">
       <c r="A146" s="2" t="n">
@@ -8601,6 +8971,7 @@
       <c r="L146" s="4" t="n"/>
       <c r="M146" s="4" t="n"/>
       <c r="N146" s="2" t="inlineStr"/>
+      <c r="P146" t="inlineStr"/>
     </row>
     <row r="147" ht="84" customHeight="1">
       <c r="A147" s="2" t="n">
@@ -8643,6 +9014,7 @@
       <c r="L147" s="4" t="n"/>
       <c r="M147" s="4" t="n"/>
       <c r="N147" s="2" t="inlineStr"/>
+      <c r="P147" t="inlineStr"/>
     </row>
     <row r="148" ht="42" customHeight="1">
       <c r="A148" s="2" t="n">
@@ -8685,6 +9057,7 @@
       <c r="L148" s="4" t="n"/>
       <c r="M148" s="4" t="n"/>
       <c r="N148" s="2" t="inlineStr"/>
+      <c r="P148" t="inlineStr"/>
     </row>
     <row r="149" ht="238" customHeight="1">
       <c r="A149" s="2" t="n">
@@ -8727,6 +9100,7 @@
       <c r="L149" s="4" t="n"/>
       <c r="M149" s="4" t="n"/>
       <c r="N149" s="2" t="inlineStr"/>
+      <c r="P149" t="inlineStr"/>
     </row>
     <row r="150" ht="42" customHeight="1">
       <c r="A150" s="2" t="n">
@@ -8769,6 +9143,7 @@
       <c r="L150" s="4" t="n"/>
       <c r="M150" s="4" t="n"/>
       <c r="N150" s="2" t="inlineStr"/>
+      <c r="P150" t="inlineStr"/>
     </row>
     <row r="151" ht="42" customHeight="1">
       <c r="A151" s="2" t="n">
@@ -8811,6 +9186,7 @@
       <c r="L151" s="4" t="n"/>
       <c r="M151" s="4" t="n"/>
       <c r="N151" s="2" t="inlineStr"/>
+      <c r="P151" t="inlineStr"/>
     </row>
     <row r="152" ht="56" customHeight="1">
       <c r="A152" s="2" t="n">
@@ -8853,6 +9229,7 @@
       <c r="L152" s="4" t="n"/>
       <c r="M152" s="4" t="n"/>
       <c r="N152" s="2" t="inlineStr"/>
+      <c r="P152" t="inlineStr"/>
     </row>
     <row r="153" ht="252" customHeight="1">
       <c r="A153" s="2" t="n">
@@ -8907,6 +9284,11 @@
           <t>G MINFLUX</t>
         </is>
       </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>wave 5 (G)</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="98" customHeight="1">
       <c r="A154" s="2" t="n">
@@ -8949,6 +9331,7 @@
       <c r="L154" s="4" t="n"/>
       <c r="M154" s="4" t="n"/>
       <c r="N154" s="2" t="inlineStr"/>
+      <c r="P154" t="inlineStr"/>
     </row>
     <row r="155" ht="70" customHeight="1">
       <c r="A155" s="2" t="n">
@@ -8991,6 +9374,7 @@
       <c r="L155" s="4" t="n"/>
       <c r="M155" s="4" t="n"/>
       <c r="N155" s="2" t="inlineStr"/>
+      <c r="P155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -9066,9 +9450,14 @@
           <t>mostly DONE; missing: several named lines per ROI</t>
         </is>
       </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O156"/>
+  <autoFilter ref="A1:P156"/>
   <dataValidations count="2">
     <dataValidation sqref="K2:K156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"work on,change,later,skip,done"</formula1>

</xml_diff>

<commit_message>
Porting list: a status column for what is done (2026-10-15)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4qGXWJdQjZ33Usauutziv
</commit_message>
<xml_diff>
--- a/docs/smap_porting/SMAP_porting_list.xlsx
+++ b/docs/smap_porting/SMAP_porting_list.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P156"/>
+  <dimension ref="A1:Q156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="7.6640625" customWidth="1" min="3" max="3"/>
@@ -550,6 +550,7 @@
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -633,6 +634,11 @@
           <t>Plan step</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Status 2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -679,7 +685,6 @@
       <c r="L2" s="4" t="n"/>
       <c r="M2" s="4" t="n"/>
       <c r="N2" s="2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -726,7 +731,6 @@
       <c r="L3" s="4" t="n"/>
       <c r="M3" s="4" t="n"/>
       <c r="N3" s="2" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -777,7 +781,6 @@
       <c r="L4" s="4" t="n"/>
       <c r="M4" s="4" t="n"/>
       <c r="N4" s="2" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" ht="56" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -828,7 +831,6 @@
       <c r="L5" s="4" t="n"/>
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="2" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -867,7 +869,6 @@
       <c r="L6" s="4" t="n"/>
       <c r="M6" s="4" t="n"/>
       <c r="N6" s="2" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -926,7 +927,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="56" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -990,6 +990,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>done (step 8): the fitters' fit region</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1036,7 +1041,6 @@
       <c r="L9" s="4" t="n"/>
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="2" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -1087,7 +1091,6 @@
       <c r="L10" s="4" t="n"/>
       <c r="M10" s="4" t="n"/>
       <c r="N10" s="2" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -1150,7 +1153,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -1213,7 +1215,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -1260,7 +1261,6 @@
       <c r="L13" s="4" t="n"/>
       <c r="M13" s="4" t="n"/>
       <c r="N13" s="2" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -1315,7 +1315,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -1366,7 +1365,6 @@
       <c r="L15" s="4" t="n"/>
       <c r="M15" s="4" t="n"/>
       <c r="N15" s="2" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -1429,7 +1427,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1476,7 +1473,6 @@
       <c r="L17" s="4" t="n"/>
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="2" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1527,7 +1523,6 @@
       <c r="L18" s="4" t="n"/>
       <c r="M18" s="4" t="n"/>
       <c r="N18" s="2" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -1574,7 +1569,6 @@
       <c r="L19" s="4" t="n"/>
       <c r="M19" s="4" t="n"/>
       <c r="N19" s="2" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1625,7 +1619,6 @@
       <c r="L20" s="4" t="n"/>
       <c r="M20" s="4" t="n"/>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1672,7 +1665,6 @@
       <c r="L21" s="4" t="n"/>
       <c r="M21" s="4" t="n"/>
       <c r="N21" s="2" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1715,7 +1707,6 @@
       <c r="L22" s="4" t="n"/>
       <c r="M22" s="4" t="n"/>
       <c r="N22" s="2" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -1782,7 +1773,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -1829,7 +1819,6 @@
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="2" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25" ht="56" customHeight="1">
       <c r="A25" s="2" t="n">
@@ -1888,7 +1877,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -1935,7 +1923,6 @@
       <c r="L26" s="4" t="n"/>
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="2" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" ht="84" customHeight="1">
       <c r="A27" s="2" t="n">
@@ -1998,7 +1985,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28" ht="56" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -2061,7 +2047,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="2" t="n">
@@ -2108,7 +2093,6 @@
       <c r="L29" s="4" t="n"/>
       <c r="M29" s="4" t="n"/>
       <c r="N29" s="2" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30" ht="56" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -2167,7 +2151,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="2" t="n">
@@ -2214,7 +2197,6 @@
       <c r="L31" s="4" t="n"/>
       <c r="M31" s="4" t="n"/>
       <c r="N31" s="2" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -2257,7 +2239,6 @@
       <c r="L32" s="4" t="n"/>
       <c r="M32" s="4" t="n"/>
       <c r="N32" s="2" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="2" t="n">
@@ -2304,7 +2285,6 @@
       <c r="L33" s="4" t="n"/>
       <c r="M33" s="4" t="n"/>
       <c r="N33" s="2" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="2" t="n">
@@ -2351,7 +2331,6 @@
       <c r="L34" s="4" t="n"/>
       <c r="M34" s="4" t="n"/>
       <c r="N34" s="2" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35" ht="70" customHeight="1">
       <c r="A35" s="2" t="n">
@@ -2412,7 +2391,12 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>wave 5 (D2)</t>
+          <t>5c</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>done (5c): Fiducials</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2459,12 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>wave 5 (D1)</t>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>done (5a): Transform, drift of another file; drift reference first/last</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2525,6 @@
           <t>D later</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -2583,7 +2571,6 @@
       <c r="L38" s="4" t="n"/>
       <c r="M38" s="4" t="n"/>
       <c r="N38" s="2" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39" ht="70" customHeight="1">
       <c r="A39" s="2" t="n">
@@ -2644,7 +2631,12 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>wave 5 (D3)</t>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>done (5d): COMET transformation over time</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2701,6 @@
           <t>C later</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41" ht="98" customHeight="1">
       <c r="A41" s="2" t="n">
@@ -2778,7 +2769,12 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>wave 5 (C1)</t>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>done (5a): Transform</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2841,12 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>wave 5 (C2/C3)</t>
+          <t>5b (+C3 later)</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>C2 done (5b): Register layers; C3 -&gt; Check overlay, with MINFLUX (topic 6)</t>
         </is>
       </c>
     </row>
@@ -2911,6 +2912,11 @@
           <t>wave 5 (C3)</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>open: Check overlay, with MINFLUX (topic 6)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="56" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -2953,7 +2959,6 @@
       <c r="L44" s="4" t="n"/>
       <c r="M44" s="4" t="n"/>
       <c r="N44" s="2" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45" ht="42" customHeight="1">
       <c r="A45" s="2" t="n">
@@ -3012,7 +3017,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46" ht="42" customHeight="1">
       <c r="A46" s="2" t="n">
@@ -3059,7 +3063,6 @@
       <c r="L46" s="4" t="n"/>
       <c r="M46" s="4" t="n"/>
       <c r="N46" s="2" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47" ht="126" customHeight="1">
       <c r="A47" s="2" t="n">
@@ -3122,7 +3125,6 @@
           <t>C later</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48" ht="56" customHeight="1">
       <c r="A48" s="2" t="n">
@@ -3187,7 +3189,12 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>wave 5 (C4)</t>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>done: Assign colours takes up to six colours</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3244,6 @@
           <t>one loader now (File/Load/Auto) with a format choice</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -3284,7 +3290,6 @@
       <c r="L50" s="4" t="n"/>
       <c r="M50" s="4" t="n"/>
       <c r="N50" s="2" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="2" t="n">
@@ -3331,7 +3336,6 @@
       <c r="L51" s="4" t="n"/>
       <c r="M51" s="4" t="n"/>
       <c r="N51" s="2" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="2" t="n">
@@ -3400,6 +3404,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>done (step 3): DECODE reader</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="2" t="n">
@@ -3468,6 +3477,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>done (step 3): Picasso reader</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="2" t="n">
@@ -3527,6 +3541,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>done (step 2): Export localizations</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="112" customHeight="1">
       <c r="A55" s="2" t="n">
@@ -3590,6 +3609,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>done (step 2)</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="2" t="n">
@@ -3649,6 +3673,11 @@
           <t>2 (optional format)</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>open: SMAP _sml.mat export, optional, later</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="2" t="n">
@@ -3695,7 +3724,6 @@
       <c r="L57" s="4" t="n"/>
       <c r="M57" s="4" t="n"/>
       <c r="N57" s="2" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
     </row>
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="2" t="n">
@@ -3746,7 +3774,6 @@
       <c r="L58" s="4" t="n"/>
       <c r="M58" s="4" t="n"/>
       <c r="N58" s="2" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3789,7 +3816,6 @@
       <c r="L59" s="4" t="n"/>
       <c r="M59" s="4" t="n"/>
       <c r="N59" s="2" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="2" t="n">
@@ -3836,7 +3862,6 @@
       <c r="L60" s="4" t="n"/>
       <c r="M60" s="4" t="n"/>
       <c r="N60" s="2" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3879,7 +3904,6 @@
       <c r="L61" s="4" t="n"/>
       <c r="M61" s="4" t="n"/>
       <c r="N61" s="2" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
     </row>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="2" t="n">
@@ -3926,7 +3950,6 @@
       <c r="L62" s="4" t="n"/>
       <c r="M62" s="4" t="n"/>
       <c r="N62" s="2" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63" ht="84" customHeight="1">
       <c r="A63" s="2" t="n">
@@ -3969,7 +3992,6 @@
       <c r="L63" s="4" t="n"/>
       <c r="M63" s="4" t="n"/>
       <c r="N63" s="2" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
     </row>
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="2" t="n">
@@ -4021,7 +4043,6 @@
           <t>moved to Analysis/Process/Layers</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr"/>
     </row>
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="2" t="n">
@@ -4068,7 +4089,6 @@
       <c r="L65" s="4" t="n"/>
       <c r="M65" s="4" t="n"/>
       <c r="N65" s="2" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
     </row>
     <row r="66" ht="56" customHeight="1">
       <c r="A66" s="2" t="n">
@@ -4135,7 +4155,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr"/>
     </row>
     <row r="67" ht="56" customHeight="1">
       <c r="A67" s="2" t="n">
@@ -4198,7 +4217,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr"/>
     </row>
     <row r="68" ht="56" customHeight="1">
       <c r="A68" s="2" t="n">
@@ -4266,7 +4284,6 @@
           <t>measuring per id: done (block over any id column); collapsing a region into one row still open, see plan J</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr"/>
     </row>
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="2" t="n">
@@ -4321,7 +4338,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr"/>
     </row>
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="2" t="n">
@@ -4386,7 +4402,12 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>wave 5 (C1)</t>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>done (5a): Transform</t>
         </is>
       </c>
     </row>
@@ -4461,6 +4482,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>done (step 9): Neighbourhood, statistic of a column</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="56" customHeight="1">
       <c r="A72" s="2" t="n">
@@ -4511,7 +4537,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr"/>
     </row>
     <row r="73" ht="84" customHeight="1">
       <c r="A73" s="2" t="n">
@@ -4554,7 +4579,6 @@
       <c r="L73" s="4" t="n"/>
       <c r="M73" s="4" t="n"/>
       <c r="N73" s="2" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="2" t="n">
@@ -4601,7 +4625,6 @@
       <c r="L74" s="4" t="n"/>
       <c r="M74" s="4" t="n"/>
       <c r="N74" s="2" t="inlineStr"/>
-      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75" ht="98" customHeight="1">
       <c r="A75" s="2" t="n">
@@ -4666,7 +4689,12 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>wave 5 (C1)</t>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>done (5a): coordinates changed, or an image layer's placement</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4743,6 @@
       <c r="L76" s="4" t="n"/>
       <c r="M76" s="4" t="n"/>
       <c r="N76" s="2" t="inlineStr"/>
-      <c r="P76" t="inlineStr"/>
     </row>
     <row r="77" ht="56" customHeight="1">
       <c r="A77" s="2" t="n">
@@ -4780,7 +4807,12 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>wave 5 (I)</t>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>done (6b): Export Stack along z</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4875,12 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>wave 5 (I)</t>
+          <t>6c</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>done (6c): Voronoi render mode</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4929,6 @@
       <c r="L79" s="4" t="n"/>
       <c r="M79" s="4" t="n"/>
       <c r="N79" s="2" t="inlineStr"/>
-      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="2" t="n">
@@ -4939,7 +4975,6 @@
       <c r="L80" s="4" t="n"/>
       <c r="M80" s="4" t="n"/>
       <c r="N80" s="2" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
     </row>
     <row r="81" ht="42" customHeight="1">
       <c r="A81" s="2" t="n">
@@ -4990,7 +5025,6 @@
       <c r="L81" s="4" t="n"/>
       <c r="M81" s="4" t="n"/>
       <c r="N81" s="2" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
     </row>
     <row r="82" ht="98" customHeight="1">
       <c r="A82" s="2" t="n">
@@ -5045,7 +5079,16 @@
           <t>I Rendering/movies</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr"/>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>6d</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>done (6d): Process image</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="2" t="n">
@@ -5092,7 +5135,6 @@
       <c r="L83" s="4" t="n"/>
       <c r="M83" s="4" t="n"/>
       <c r="N83" s="2" t="inlineStr"/>
-      <c r="P83" t="inlineStr"/>
     </row>
     <row r="84" ht="42" customHeight="1">
       <c r="A84" s="2" t="n">
@@ -5139,7 +5181,6 @@
       <c r="L84" s="4" t="n"/>
       <c r="M84" s="4" t="n"/>
       <c r="N84" s="2" t="inlineStr"/>
-      <c r="P84" t="inlineStr"/>
     </row>
     <row r="85" ht="42" customHeight="1">
       <c r="A85" s="2" t="n">
@@ -5190,7 +5231,6 @@
       <c r="L85" s="4" t="n"/>
       <c r="M85" s="4" t="n"/>
       <c r="N85" s="2" t="inlineStr"/>
-      <c r="P85" t="inlineStr"/>
     </row>
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="2" t="n">
@@ -5237,7 +5277,6 @@
       <c r="L86" s="4" t="n"/>
       <c r="M86" s="4" t="n"/>
       <c r="N86" s="2" t="inlineStr"/>
-      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87" ht="56" customHeight="1">
       <c r="A87" s="2" t="n">
@@ -5310,6 +5349,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>done (step 4): Measure/Histogram</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="56" customHeight="1">
       <c r="A88" s="2" t="n">
@@ -5381,6 +5425,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>done (step 5): Measure/Time Course</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="28" customHeight="1">
       <c r="A89" s="2" t="n">
@@ -5441,7 +5490,12 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>wave 5 (A6)</t>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>done (5e): Stability, vibrations</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5544,6 @@
       <c r="L90" s="4" t="n"/>
       <c r="M90" s="4" t="n"/>
       <c r="N90" s="2" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
     </row>
     <row r="91" ht="98" customHeight="1">
       <c r="A91" s="2" t="n">
@@ -5547,7 +5600,12 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>17a-c</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>done (17a-c): Spatial statistics</t>
         </is>
       </c>
     </row>
@@ -5626,6 +5684,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>done (step 10): Find clusters</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="98" customHeight="1">
       <c r="A93" s="2" t="n">
@@ -5690,7 +5753,12 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>17a</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>done (17a, 12): Spatial statistics; Cluster shape</t>
         </is>
       </c>
     </row>
@@ -5761,6 +5829,11 @@
           <t>9 + 10</t>
         </is>
       </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>done (9, 10): Voronoi density, Voronoi clusters</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="84" customHeight="1">
       <c r="A95" s="2" t="n">
@@ -5833,6 +5906,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>done (step 9)</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="70" customHeight="1">
       <c r="A96" s="2" t="n">
@@ -5905,6 +5983,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>done (step 7): Shuffle ids</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="42" customHeight="1">
       <c r="A97" s="2" t="n">
@@ -5981,6 +6064,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>done (step 12): Cluster shape</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -6023,7 +6111,6 @@
       <c r="L98" s="4" t="n"/>
       <c r="M98" s="4" t="n"/>
       <c r="N98" s="2" t="inlineStr"/>
-      <c r="P98" t="inlineStr"/>
     </row>
     <row r="99" ht="112" customHeight="1">
       <c r="A99" s="2" t="n">
@@ -6096,6 +6183,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>partly (step 18): Blinking per region; the counting fit later, on the NPC model</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="70" customHeight="1">
       <c r="A100" s="2" t="n">
@@ -6138,7 +6230,6 @@
       <c r="L100" s="4" t="n"/>
       <c r="M100" s="4" t="n"/>
       <c r="N100" s="2" t="inlineStr"/>
-      <c r="P100" t="inlineStr"/>
     </row>
     <row r="101" ht="126" customHeight="1">
       <c r="A101" s="2" t="n">
@@ -6208,7 +6299,12 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>19a</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>done (19a): Link tracks</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6376,12 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>19c</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>done (19c): MSD, jump distances; step finding and the motor analysis later</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6430,6 @@
       <c r="L103" s="4" t="n"/>
       <c r="M103" s="4" t="n"/>
       <c r="N103" s="2" t="inlineStr"/>
-      <c r="P103" t="inlineStr"/>
     </row>
     <row r="104" ht="126" customHeight="1">
       <c r="A104" s="2" t="n">
@@ -6466,6 +6566,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>done (step 11)</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="42" customHeight="1">
       <c r="A106" s="2" t="n">
@@ -6534,6 +6639,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>done (step 11)</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="2" t="n">
@@ -6602,6 +6712,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>done (step 14)</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="2" t="n">
@@ -6668,6 +6783,11 @@
       <c r="P108" t="inlineStr">
         <is>
           <t>14</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>done (step 14)</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6849,6 @@
           <t>mostly there: Column to ROIs on filenumber</t>
         </is>
       </c>
-      <c r="P109" t="inlineStr"/>
     </row>
     <row r="110" ht="56" customHeight="1">
       <c r="A110" s="2" t="n">
@@ -6802,6 +6921,11 @@
           <t>11 (later preset)</t>
         </is>
       </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>open: a later preset of Segment regions</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="2" t="n">
@@ -6848,7 +6972,6 @@
       <c r="L111" s="4" t="n"/>
       <c r="M111" s="4" t="n"/>
       <c r="N111" s="2" t="inlineStr"/>
-      <c r="P111" t="inlineStr"/>
     </row>
     <row r="112" ht="98" customHeight="1">
       <c r="A112" s="2" t="n">
@@ -6915,6 +7038,11 @@
       <c r="P112" t="inlineStr">
         <is>
           <t>11 (later presets)</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>open: later presets</t>
         </is>
       </c>
     </row>
@@ -6968,7 +7096,6 @@
           <t>Localization Statistics is per_region now</t>
         </is>
       </c>
-      <c r="P113" t="inlineStr"/>
     </row>
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="2" t="n">
@@ -7020,7 +7147,6 @@
           <t>moved to Analysis/Measure/NPC Corners (per_region)</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr"/>
     </row>
     <row r="115" ht="42" customHeight="1">
       <c r="A115" s="2" t="n">
@@ -7160,6 +7286,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>done (step 15): Circle fit</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="56" customHeight="1">
       <c r="A117" s="2" t="n">
@@ -7232,6 +7363,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>done (step 15): Centre ROIs</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="70" customHeight="1">
       <c r="A118" s="2" t="n">
@@ -7376,6 +7512,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>done (step 15)</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="112" customHeight="1">
       <c r="A120" s="2" t="n">
@@ -7440,7 +7581,12 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>17 (+ C2)</t>
+          <t>17c (+5b)</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>done (17c, 5b)</t>
         </is>
       </c>
     </row>
@@ -7511,6 +7657,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>done (step 12)</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="28" customHeight="1">
       <c r="A122" s="2" t="n">
@@ -7579,6 +7730,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>done (step 18): Blinking</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="28" customHeight="1">
       <c r="A123" s="2" t="n">
@@ -7629,7 +7785,6 @@
       <c r="L123" s="4" t="n"/>
       <c r="M123" s="4" t="n"/>
       <c r="N123" s="2" t="inlineStr"/>
-      <c r="P123" t="inlineStr"/>
     </row>
     <row r="124" ht="42" customHeight="1">
       <c r="A124" s="2" t="n">
@@ -7680,7 +7835,6 @@
       <c r="L124" s="4" t="n"/>
       <c r="M124" s="4" t="n"/>
       <c r="N124" s="2" t="inlineStr"/>
-      <c r="P124" t="inlineStr"/>
     </row>
     <row r="125" ht="140" customHeight="1">
       <c r="A125" s="2" t="n">
@@ -7739,7 +7893,6 @@
           <t>J Later</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr"/>
     </row>
     <row r="126" ht="28" customHeight="1">
       <c r="A126" s="2" t="n">
@@ -7791,7 +7944,6 @@
           <t>blocks of a chain now</t>
         </is>
       </c>
-      <c r="P126" t="inlineStr"/>
     </row>
     <row r="127" ht="28" customHeight="1">
       <c r="A127" s="2" t="n">
@@ -7838,7 +7990,6 @@
       <c r="L127" s="4" t="n"/>
       <c r="M127" s="4" t="n"/>
       <c r="N127" s="2" t="inlineStr"/>
-      <c r="P127" t="inlineStr"/>
     </row>
     <row r="128" ht="42" customHeight="1">
       <c r="A128" s="2" t="n">
@@ -7906,7 +8057,6 @@
           <t>DONE: Analysis/Regions/Filter ROIs</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -7974,7 +8124,6 @@
           <t>DONE: Analysis/Regions/Sort ROIs</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -8039,6 +8188,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>done (step 14)</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="70" customHeight="1">
       <c r="A131" s="2" t="n">
@@ -8115,6 +8269,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>done (step 6): Export table</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="56" customHeight="1">
       <c r="A132" s="2" t="n">
@@ -8186,7 +8345,6 @@
           <t>DONE: Analysis/Regions/Regions to column (roi_id too), block write values</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr"/>
     </row>
     <row r="133" ht="56" customHeight="1">
       <c r="A133" s="2" t="n">
@@ -8390,6 +8548,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>done (step 16): Average ROIs</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -8444,7 +8607,6 @@
           <t>E1 ROI housekeeping</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr"/>
     </row>
     <row r="137" ht="28" customHeight="1">
       <c r="A137" s="2" t="n">
@@ -8491,7 +8653,6 @@
       <c r="L137" s="4" t="n"/>
       <c r="M137" s="4" t="n"/>
       <c r="N137" s="2" t="inlineStr"/>
-      <c r="P137" t="inlineStr"/>
     </row>
     <row r="138" ht="266" customHeight="1">
       <c r="A138" s="2" t="n">
@@ -8538,7 +8699,6 @@
       <c r="L138" s="4" t="n"/>
       <c r="M138" s="4" t="n"/>
       <c r="N138" s="2" t="inlineStr"/>
-      <c r="P138" t="inlineStr"/>
     </row>
     <row r="139" ht="210" customHeight="1">
       <c r="A139" s="2" t="n">
@@ -8675,7 +8835,12 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>wave 5 (I)</t>
+          <t>6b (+topic 4)</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>MovieRunningWindow done (6b); mkMovieByFilter -&gt; figures of regions (topic 4)</t>
         </is>
       </c>
     </row>
@@ -8742,7 +8907,12 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>wave 5 (I)</t>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>done (6b): raw frames beside the view</t>
         </is>
       </c>
     </row>
@@ -8801,7 +8971,12 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>19b, 6b</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>done (6b): tracks with a tail in Export Stack; co-tracking with MINFLUX (topic 6)</t>
         </is>
       </c>
     </row>
@@ -8846,7 +9021,6 @@
       <c r="L143" s="4" t="n"/>
       <c r="M143" s="4" t="n"/>
       <c r="N143" s="2" t="inlineStr"/>
-      <c r="P143" t="inlineStr"/>
     </row>
     <row r="144" ht="42" customHeight="1">
       <c r="A144" s="2" t="n">
@@ -8889,7 +9063,6 @@
       <c r="L144" s="4" t="n"/>
       <c r="M144" s="4" t="n"/>
       <c r="N144" s="2" t="inlineStr"/>
-      <c r="P144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
@@ -8928,7 +9101,6 @@
       <c r="L145" s="4" t="n"/>
       <c r="M145" s="4" t="n"/>
       <c r="N145" s="2" t="inlineStr"/>
-      <c r="P145" t="inlineStr"/>
     </row>
     <row r="146" ht="28" customHeight="1">
       <c r="A146" s="2" t="n">
@@ -8971,7 +9143,6 @@
       <c r="L146" s="4" t="n"/>
       <c r="M146" s="4" t="n"/>
       <c r="N146" s="2" t="inlineStr"/>
-      <c r="P146" t="inlineStr"/>
     </row>
     <row r="147" ht="84" customHeight="1">
       <c r="A147" s="2" t="n">
@@ -9014,7 +9185,6 @@
       <c r="L147" s="4" t="n"/>
       <c r="M147" s="4" t="n"/>
       <c r="N147" s="2" t="inlineStr"/>
-      <c r="P147" t="inlineStr"/>
     </row>
     <row r="148" ht="42" customHeight="1">
       <c r="A148" s="2" t="n">
@@ -9057,7 +9227,6 @@
       <c r="L148" s="4" t="n"/>
       <c r="M148" s="4" t="n"/>
       <c r="N148" s="2" t="inlineStr"/>
-      <c r="P148" t="inlineStr"/>
     </row>
     <row r="149" ht="238" customHeight="1">
       <c r="A149" s="2" t="n">
@@ -9100,7 +9269,6 @@
       <c r="L149" s="4" t="n"/>
       <c r="M149" s="4" t="n"/>
       <c r="N149" s="2" t="inlineStr"/>
-      <c r="P149" t="inlineStr"/>
     </row>
     <row r="150" ht="42" customHeight="1">
       <c r="A150" s="2" t="n">
@@ -9143,7 +9311,6 @@
       <c r="L150" s="4" t="n"/>
       <c r="M150" s="4" t="n"/>
       <c r="N150" s="2" t="inlineStr"/>
-      <c r="P150" t="inlineStr"/>
     </row>
     <row r="151" ht="42" customHeight="1">
       <c r="A151" s="2" t="n">
@@ -9186,7 +9353,6 @@
       <c r="L151" s="4" t="n"/>
       <c r="M151" s="4" t="n"/>
       <c r="N151" s="2" t="inlineStr"/>
-      <c r="P151" t="inlineStr"/>
     </row>
     <row r="152" ht="56" customHeight="1">
       <c r="A152" s="2" t="n">
@@ -9229,7 +9395,6 @@
       <c r="L152" s="4" t="n"/>
       <c r="M152" s="4" t="n"/>
       <c r="N152" s="2" t="inlineStr"/>
-      <c r="P152" t="inlineStr"/>
     </row>
     <row r="153" ht="252" customHeight="1">
       <c r="A153" s="2" t="n">
@@ -9331,7 +9496,6 @@
       <c r="L154" s="4" t="n"/>
       <c r="M154" s="4" t="n"/>
       <c r="N154" s="2" t="inlineStr"/>
-      <c r="P154" t="inlineStr"/>
     </row>
     <row r="155" ht="70" customHeight="1">
       <c r="A155" s="2" t="n">
@@ -9374,7 +9538,6 @@
       <c r="L155" s="4" t="n"/>
       <c r="M155" s="4" t="n"/>
       <c r="N155" s="2" t="inlineStr"/>
-      <c r="P155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -9453,6 +9616,11 @@
       <c r="P156" t="inlineStr">
         <is>
           <t>13</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>done (step 13)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Porting list: a status column for 2026-10-25
What has landed since 2026-10-15 (Filter / Sort ROIs, Regions to column,
Combine files, ROI images, the MINFLUX reader and MBM tools, uiPSF v2) and
what comes next: beads, CME patches and positions from a file as methods
of Segment regions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WRpoGmgakV2YKdiNHp5LUL
</commit_message>
<xml_diff>
--- a/docs/smap_porting/SMAP_porting_list.xlsx
+++ b/docs/smap_porting/SMAP_porting_list.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q156"/>
+  <dimension ref="A1:R156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="7.6640625" customWidth="1" min="3" max="3"/>
@@ -551,6 +551,7 @@
     <col width="45" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -639,6 +640,11 @@
           <t>Status 2026-10-15</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Status 2026-10-25</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -1877,6 +1883,11 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>in progress: uiPSF v2 in PyTorch (src/uipsf), its own plan in docs/uipsf</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -1985,6 +1996,11 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>partly: Spline 3D's focus in the sample (calibrate/depth.py, uipsf's pupil drawn at depth); a z-correction map from beads in gel still open</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="56" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -2847,6 +2863,11 @@
       <c r="Q42" t="inlineStr">
         <is>
           <t>C2 done (5b): Register layers; C3 -&gt; Check overlay, with MINFLUX (topic 6)</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>C2 done (5b); C3 still open (Check overlay, with MINFLUX)</t>
         </is>
       </c>
     </row>
@@ -4155,6 +4176,11 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>done: Analysis/Process/Combine files (frames and time continued, ids kept apart)</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="56" customHeight="1">
       <c r="A67" s="2" t="n">
@@ -6188,6 +6214,11 @@
           <t>partly (step 18): Blinking per region; the counting fit later, on the NPC model</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>partly: Blinking per region (step 18); the counting fit still open</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="70" customHeight="1">
       <c r="A100" s="2" t="n">
@@ -6496,6 +6527,11 @@
       <c r="P104" t="inlineStr">
         <is>
           <t>wave 5 (G)</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>partly: Abberior .msr reader, MBM drift and registration, tid as an id column for Tracking analysis; the stepping and dual-track tools still open</t>
         </is>
       </c>
     </row>
@@ -6926,6 +6962,11 @@
           <t>open: a later preset of Segment regions</t>
         </is>
       </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>next: a beads method of Segment regions, on Fiducials' find_beads (in design 2026-10-25)</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="2" t="n">
@@ -7043,6 +7084,11 @@
       <c r="Q112" t="inlineStr">
         <is>
           <t>open: later presets</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>next: a patches method of Segment regions with a CME preset (in design 2026-10-25); cells, fibrils skipped</t>
         </is>
       </c>
     </row>
@@ -7214,6 +7260,11 @@
           <t>wave 5 (H/E5)</t>
         </is>
       </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>open: decide with LocMoFit (H)</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="42" customHeight="1">
       <c r="A116" s="2" t="n">
@@ -7440,6 +7491,11 @@
           <t>wave 5 (H)</t>
         </is>
       </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>open: port or Weiqing's approach, undecided</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="84" customHeight="1">
       <c r="A119" s="2" t="n">
@@ -7891,6 +7947,11 @@
       <c r="N125" s="2" t="inlineStr">
         <is>
           <t>J Later</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>open: image intensity at localizations / ROIs likely needed</t>
         </is>
       </c>
     </row>
@@ -8057,6 +8118,11 @@
           <t>DONE: Analysis/Regions/Filter ROIs</t>
         </is>
       </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>done: Analysis/Regions/Filter ROIs</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -8124,6 +8190,11 @@
           <t>DONE: Analysis/Regions/Sort ROIs</t>
         </is>
       </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>done: Analysis/Regions/Sort ROIs</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -8345,6 +8416,11 @@
           <t>DONE: Analysis/Regions/Regions to column (roi_id too), block write values</t>
         </is>
       </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>done: Analysis/Regions/Regions to column (roi_id, any value)</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="56" customHeight="1">
       <c r="A133" s="2" t="n">
@@ -8413,6 +8489,11 @@
           <t>wave 5 (E6)</t>
         </is>
       </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>done: File/Export/ROI images (PDF gallery at one scale, turned by a named line, values as titles)</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="70" customHeight="1">
       <c r="A134" s="2" t="n">
@@ -8476,6 +8557,11 @@
           <t>wave 5 (E6)</t>
         </is>
       </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>mostly done: ROI images as a TIFF stack; single TIFFs per ROI and 3D volumes not</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="98" customHeight="1">
       <c r="A135" s="2" t="n">
@@ -8607,6 +8693,11 @@
           <t>E1 ROI housekeeping</t>
         </is>
       </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>next: positions from a file as a method of Segment regions (with 109, 111)</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="28" customHeight="1">
       <c r="A137" s="2" t="n">
@@ -8771,6 +8862,11 @@
           <t>wave 5 (H)</t>
         </is>
       </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>open: see #117</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="56" customHeight="1">
       <c r="A140" s="2" t="n">
@@ -8843,6 +8939,11 @@
           <t>MovieRunningWindow done (6b); mkMovieByFilter -&gt; figures of regions (topic 4)</t>
         </is>
       </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>done: MovieRunningWindow (6b); the player and view path (smappy.scan); mkMovieByFilter not</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="42" customHeight="1">
       <c r="A141" s="2" t="n">
@@ -9452,6 +9553,11 @@
       <c r="P153" t="inlineStr">
         <is>
           <t>wave 5 (G)</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>partly: see #103; MINFLUX analysis plugins still to be decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Survey and porting tables: what was built and decided on 2026-10-28
Survey #4 (COMET weights), qPAINT, #59-#61 (watcher, summary page, time
trace), #67 (session restore) done; #56 parallel files not wanted;
#57 already there; #66 plugin registry later.  Porting list #66-#68 done
(a Status 2026-10-28 column in the spreadsheet).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/smap_porting/SMAP_porting_list.xlsx
+++ b/docs/smap_porting/SMAP_porting_list.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R156"/>
+  <dimension ref="A1:S156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="7.6640625" customWidth="1" min="3" max="3"/>
@@ -552,6 +552,7 @@
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="60" customWidth="1" min="17" max="17"/>
     <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -645,6 +646,11 @@
           <t>Status 2026-10-25</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Status 2026-10-28</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -4243,6 +4249,11 @@
           <t>J Later</t>
         </is>
       </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>done: Collapse by id (Analysis/Process), the compact form -- one row per blink, mainly a smaller file; writing grouped values into member rows declined</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="56" customHeight="1">
       <c r="A68" s="2" t="n">
@@ -4310,6 +4321,11 @@
           <t>measuring per id: done (block over any id column); collapsing a region into one row still open, see plan J</t>
         </is>
       </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>done: Collapse by id keyed by any id column (group_id, track_id, cluster_id, ...)</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="2" t="n">
@@ -4362,6 +4378,11 @@
       <c r="N69" s="2" t="inlineStr">
         <is>
           <t>J Later</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>done: Edit columns (Analysis/Process) renames or removes; Save smappy HDF5 has a columns choice</t>
         </is>
       </c>
     </row>

</xml_diff>